<commit_message>
Corte SD: una S02 mas, entregada dentro de la ventana de tarde
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S04-corte-12sep.xlsx
+++ b/calificaciones/P00-S04-corte-12sep.xlsx
@@ -746,31 +746,31 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
           <t>—</t>
@@ -778,7 +778,7 @@
       </c>
       <c r="I8" s="10" t="inlineStr">
         <is>
-          <t>Ya hiciste tu primer push. Falta toda la S02.</t>
+          <t>Completa. Llego tarde pero dentro de la ventana, y esta bien hecha: no te falta nada de la S02.</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
     <row r="54">
       <c r="A54" s="15" t="inlineStr">
         <is>
-          <t>S02 completa: 37 / 43   ·   parcial: 2   ·   sin entregar: 4</t>
+          <t>S02 completa: 38 / 43   ·   parcial: 2   ·   sin entregar: 3</t>
         </is>
       </c>
     </row>

</xml_diff>